<commit_message>
Test lại các testcase fail, kiểm thử tính năng Quên mật khẩu
</commit_message>
<xml_diff>
--- a/TestReport_CMS.xlsx
+++ b/TestReport_CMS.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QuanLyKhoaHoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBFFFF8-B219-47D9-9942-4669712FF8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFECA10-B68E-4056-BCD8-BD5CF7D7AE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="821" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="821" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="97" r:id="rId1"/>
-    <sheet name="Module Login" sheetId="123" r:id="rId2"/>
-    <sheet name="Module Register" sheetId="122" r:id="rId3"/>
+    <sheet name="Module Register" sheetId="122" r:id="rId2"/>
+    <sheet name="Module Login" sheetId="123" r:id="rId3"/>
     <sheet name="Test Report" sheetId="107" r:id="rId4"/>
   </sheets>
   <externalReferences>
@@ -53,7 +53,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="6">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -68,20 +68,60 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="6">
     <bk>
       <rc t="1" v="0"/>
     </bk>
     <bk>
       <rc t="1" v="1"/>
     </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="100">
   <si>
     <t>TC1</t>
   </si>
@@ -246,9 +286,6 @@
     <t>Commit 3826ff4 - Đăng kí tài khoản học viên, đăng nhập (PR #1)</t>
   </si>
   <si>
-    <t>Viết 8 test case cho chức năng Đăng ký và 5 test case cho chức năng Đăng nhập</t>
-  </si>
-  <si>
     <t>Test Case Document</t>
   </si>
   <si>
@@ -267,48 +304,6 @@
     <t>1: Nhập thông tin tên và mật khẩu hợp lệ
 2: Nhập email giả định dạng "nguyenvana@1.2"
 3: Nhấn nút 'Đăng ký'</t>
-  </si>
-  <si>
-    <r>
-      <t>Hiển thị cảnh báo lỗi 
-"</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Tahoma"/>
-        <family val="2"/>
-      </rPr>
-      <t>Mật khẩu phải từ 8-16 ký tự, có chữ hoa, chữ thường, số và ký tự đặc biệt.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Tahoma"/>
-        <family val="2"/>
-      </rPr>
-      <t>"</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Hiển thị cảnh báo lỗi
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Tahoma"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Email không hợp lệ."</t>
-    </r>
   </si>
   <si>
     <r>
@@ -434,13 +429,152 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">1: Nhập thông tin tên và email hợp lệ
+2: Nhập mật khẩu đúng nhưng có chứa khoảng trắng ' ' ở đầu hoặc cuối mật khẩu
+3: Chọn đúng vai trò tài khoản
+4: Nhấn nút "Đăng nhập"
+</t>
+  </si>
+  <si>
+    <t>1: Nhập thông tin tên và email hợp lệ 
+2: Chọn đúng vai trò người dùng
+3: Nhập sai mật khẩu
+4: Nhấn nút "Đăng nhập"
+5: Lặp lại các bước trên 5 lần</t>
+  </si>
+  <si>
+    <t>1. Kiểm tra đăng nhập với mật khẩu chứa khoảng trắng</t>
+  </si>
+  <si>
+    <t>CMS_18</t>
+  </si>
+  <si>
+    <t>Thành Nhật</t>
+  </si>
+  <si>
+    <t>28/03/2025</t>
+  </si>
+  <si>
+    <t>1: Nhập thông tin tên và mật khẩu hợp lệ
+2: Nhập email giả định dạng "abc@1.2"
+3: Nhấn nút 'Đăng ký'</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>bảo mật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chức năng Đăng nhập tài khoản  khi người dùng nhập sai mật khẩu nhiều lần</t>
+    </r>
+  </si>
+  <si>
+    <t>27/03/2025</t>
+  </si>
+  <si>
+    <t>2. Kiểm tra đăng nhập sai mật khẩu nhiều lần</t>
+  </si>
+  <si>
+    <t>Hiển thị cảnh báo nhập sai mật khẩu nhiều lần, yêu cầu đặt lại mật khẩu</t>
+  </si>
+  <si>
+    <t>3. Kiểm tra quên mật khẩu khi gửi nhiều yêu cầu đặt lại cho 1 email</t>
+  </si>
+  <si>
+    <t>1. Chọn tính năng Quên mật khẩu
+2. Nhập email hợp lệ có trong hệ thống
+3. Nhấn nút "Gửi OTP"
+4. Không nhập OTP
+5. Lặp lại bước 2 đến 4 thêm 4 lần</t>
+  </si>
+  <si>
+    <t>Fail lần 1</t>
+  </si>
+  <si>
+    <t>TC4</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>bảo mật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chức năng Đăng nhập tính năng Quên mật khẩu khi gửi nhiều yêu cầu đặt lại trong thời gian ngắn cho 1 email</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>bảo mật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chức năng Đăng nhập tính năng Quên mật khẩu khi dùng mã OTP đã nhận được ở ở lần trước thử cho lần sau</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Chọn tính năng Quên mật khẩu
+2. Nhập email hợp lệ có trong hệ thống
+3. Nhấn nút "Gửi OTP"
+4. Không nhập OTP
+5. Lặp lại bước 2 đến 4 thêm 1 lần
+6. Lấy mã OTP lần nhận đầu tiên nhập cho lần này</t>
+  </si>
+  <si>
+    <t>Hiển thị cảnh báo lỗi
+"Mã OTP không chính xác. Vui lòng thử lại."</t>
+  </si>
+  <si>
     <r>
       <t>Hiển thị cảnh báo lỗi 
 "</t>
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Tahoma"/>
@@ -450,7 +584,6 @@
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="10"/>
         <color indexed="8"/>
         <rFont val="Tahoma"/>
@@ -460,33 +593,172 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1: Nhập thông tin tên và email hợp lệ
-2: Nhập mật khẩu đúng nhưng có chứa khoảng trắng ' ' ở đầu hoặc cuối mật khẩu
-3: Chọn đúng vai trò tài khoản
-4: Nhấn nút "Đăng nhập"
-</t>
-  </si>
-  <si>
-    <t>Test case dùng để kiểm thử chức năng Đăng nhập tài khoản  khi người dùng nhập sai mật khẩu nhiều lần</t>
-  </si>
-  <si>
-    <t>1: Nhập thông tin tên và email hợp lệ 
-2: Chọn đúng vai trò người dùng
-3: Nhập sai mật khẩu
-4: Nhấn nút "Đăng nhập"
-5: Lặp lại các bước trên 5 lần</t>
-  </si>
-  <si>
-    <t>Hiển thị cảnh báo nhập sai mật khẩu nhiều lần, khóa tài khoản trong 1 khoảng thời gian</t>
-  </si>
-  <si>
-    <t>1. Kiểm tra đăng nhập với mật khẩu chứa khoảng trắng</t>
-  </si>
-  <si>
-    <t>2. Kiểm tra khóa tài khoản khi nhập sai mật khẩu nhiều lần</t>
-  </si>
-  <si>
-    <t>CMS_18</t>
+    <t>Hiển thị cảnh báo 
+"Quá nhiều yêu cầu, vui lòng thử lại sau X phút"</t>
+  </si>
+  <si>
+    <t>Hiển thị cảnh báo lỗi
+"Email không hợp lệ."</t>
+  </si>
+  <si>
+    <r>
+      <t>Hiển thị cảnh báo lỗi 
+"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mật khẩu phải từ 8-16 ký tự, có chữ hoa, chữ thường, số và ký tự đặc biệt.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>4. Kiểm tra quên mật khẩu khi dùng mã OTP của phiên khác đặt lại mật khẩu cho phiên này</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>bảo mật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chức năng Đăng nhập tính năng Quên mật khẩu khi dùng mã OTP hết hạn để đổi mật khẩu.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Chọn tính năng Quên mật khẩu
+2. Nhập email hợp lệ có trong hệ thống
+3. Nhấn nút "Gửi OTP"
+4. Không nhập OTP
+5. Chỉnh thời gian sang 24h sau
+6. Nhập mã OTP vào hệ thống</t>
+  </si>
+  <si>
+    <t>Hiển thị cảnh báo lỗi
+"Mã OTP đã hết hạn. Vui lòng yêu cầu lại."</t>
+  </si>
+  <si>
+    <t>Commit 0539dfa - Cập nhật đăng kí, đăng nhập, hiển thị khóa học, giỏ hàng, cấu hình mysql (PR #3)</t>
+  </si>
+  <si>
+    <t>. Viết 8 test case cho chức năng Đăng ký
+. Viết 5 test case cho chức năng Đăng nhập
+. Tiến hành test và ghi nhận kết quả 22/03</t>
+  </si>
+  <si>
+    <t>. Cập nhật kết quả test lại 1 số test case fail
+. Viết 7 test case cho chức năng Quên mật khẩu
+. Tiến hành test và ghi nhận kết quả 28/03</t>
+  </si>
+  <si>
+    <t>System Name：</t>
+  </si>
+  <si>
+    <t>Module Code：</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử lại </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>bảo mật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chức năng Đăng nhập tài khoản  khi người dùng nhập sai mật khẩu nhiều lần</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử lại </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>chức năng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Đăng kí tài khoản cho học viên khi người dùng nhập sai định dạng email - email không tồn tại</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Test case dùng để kiểm thử lại </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>chức năng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Đăng kí tài khoản cho học viên khi người dùng nhập mật khẩu chứa khoảng trắng ' '</t>
+    </r>
+  </si>
+  <si>
+    <t>5. Kiểm tra quên mật khẩu khi dùng mã OTP hết hạn để đổi mật khẩu</t>
+  </si>
+  <si>
+    <t>TC5</t>
   </si>
 </sst>
 </file>
@@ -497,7 +769,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -600,11 +872,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
@@ -635,13 +902,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
@@ -654,8 +914,13 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -692,6 +957,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="35">
     <border>
@@ -1160,7 +1431,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1219,16 +1490,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1318,9 +1579,6 @@
     <xf numFmtId="1" fontId="6" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1345,9 +1603,6 @@
     <xf numFmtId="15" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1357,9 +1612,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1371,9 +1626,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1398,12 +1650,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="15" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1416,102 +1662,128 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="15" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="30" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="31" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="27" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="30" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="30" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="30" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="31" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="27" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1519,21 +1791,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1610,13 +1867,29 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
   <rv s="0">
     <v>0</v>
     <v>5</v>
   </rv>
   <rv s="0">
     <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -1635,6 +1908,10 @@
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
   <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
 </richValueRels>
 </file>
 
@@ -1932,7 +2209,7 @@
     <col min="2" max="2" width="14.109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="1"/>
     <col min="4" max="4" width="15" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.77734375" style="1" customWidth="1"/>
     <col min="7" max="7" width="20.44140625" style="1" customWidth="1"/>
     <col min="8" max="8" width="26.6640625" style="1" customWidth="1"/>
@@ -1955,7 +2232,7 @@
       <c r="B3" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="61">
+      <c r="C3" s="57">
         <v>1</v>
       </c>
       <c r="D3" s="28"/>
@@ -2004,7 +2281,7 @@
         <v>35</v>
       </c>
       <c r="C7" s="104" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D7" s="104"/>
       <c r="E7" s="105"/>
@@ -2034,148 +2311,164 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="34" customFormat="1" ht="26.4">
-      <c r="B11" s="50" t="s">
+    <row r="11" spans="1:8" s="30" customFormat="1" ht="26.4">
+      <c r="B11" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="51" t="s">
+      <c r="D11" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="51" t="s">
+      <c r="E11" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="51" t="s">
+      <c r="F11" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="52" t="s">
+      <c r="G11" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="86" t="s">
+      <c r="H11" s="79" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="34" customFormat="1" ht="39.6">
-      <c r="B12" s="36" t="s">
+    <row r="12" spans="1:8" s="30" customFormat="1" ht="43.2" customHeight="1">
+      <c r="B12" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="103" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="102" t="s">
+      <c r="D12" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="73" t="s">
+      <c r="E12" s="92" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="85"/>
-      <c r="H12" s="87" t="s">
+      <c r="G12" s="95" t="s">
+        <v>67</v>
+      </c>
+      <c r="H12" s="80" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="34" customFormat="1">
-      <c r="B13" s="98"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="73"/>
-      <c r="G13" s="97"/>
-      <c r="H13" s="87"/>
-    </row>
-    <row r="14" spans="1:8" s="35" customFormat="1" ht="13.2">
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="73"/>
-      <c r="G14" s="97"/>
-      <c r="H14" s="87"/>
-    </row>
-    <row r="15" spans="1:8" s="35" customFormat="1" ht="13.2">
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="42"/>
-    </row>
-    <row r="16" spans="1:8" s="34" customFormat="1">
-      <c r="B16" s="36"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="45"/>
-    </row>
-    <row r="17" spans="2:8" s="34" customFormat="1">
-      <c r="B17" s="43"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="42"/>
-    </row>
-    <row r="18" spans="2:8" s="34" customFormat="1">
-      <c r="B18" s="43"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-    </row>
-    <row r="19" spans="2:8" s="34" customFormat="1">
-      <c r="B19" s="43"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="42"/>
-    </row>
-    <row r="20" spans="2:8" s="34" customFormat="1">
-      <c r="B20" s="43"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="42"/>
-    </row>
-    <row r="21" spans="2:8" s="34" customFormat="1">
-      <c r="B21" s="43"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
-    </row>
-    <row r="22" spans="2:8" s="34" customFormat="1">
-      <c r="B22" s="43"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="42"/>
-    </row>
-    <row r="23" spans="2:8" s="34" customFormat="1">
-      <c r="B23" s="46"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="49"/>
+    <row r="13" spans="1:8" s="30" customFormat="1" ht="67.8" customHeight="1">
+      <c r="B13" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="93" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="92" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="68" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="80" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="31" customFormat="1" ht="13.2">
+      <c r="B14" s="32"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="68"/>
+      <c r="G14" s="88"/>
+      <c r="H14" s="80"/>
+    </row>
+    <row r="15" spans="1:8" s="31" customFormat="1" ht="13.2">
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
+    </row>
+    <row r="16" spans="1:8" s="30" customFormat="1">
+      <c r="B16" s="32"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="41"/>
+    </row>
+    <row r="17" spans="2:8" s="30" customFormat="1">
+      <c r="B17" s="39"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="38"/>
+    </row>
+    <row r="18" spans="2:8" s="30" customFormat="1">
+      <c r="B18" s="39"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="38"/>
+    </row>
+    <row r="19" spans="2:8" s="30" customFormat="1">
+      <c r="B19" s="39"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="38"/>
+    </row>
+    <row r="20" spans="2:8" s="30" customFormat="1">
+      <c r="B20" s="39"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="38"/>
+    </row>
+    <row r="21" spans="2:8" s="30" customFormat="1">
+      <c r="B21" s="39"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
+    </row>
+    <row r="22" spans="2:8" s="30" customFormat="1">
+      <c r="B22" s="39"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
+    </row>
+    <row r="23" spans="2:8" s="30" customFormat="1">
+      <c r="B23" s="42"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2192,7 +2485,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F6884C4-AFEC-4BBC-9DC8-80B5528C1C8F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2205,302 +2498,364 @@
     <col min="6" max="6" width="23.6640625" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="17.109375" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" style="93"/>
-    <col min="10" max="10" width="18" style="92" customWidth="1"/>
+    <col min="9" max="9" width="9" style="86"/>
+    <col min="10" max="10" width="18" style="85" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
-      <c r="I1" s="99"/>
+      <c r="I1" s="90"/>
       <c r="J1" s="6"/>
       <c r="K1" s="7"/>
     </row>
     <row r="2" spans="1:11" s="2" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
       <c r="A2" s="7"/>
-      <c r="B2" s="132"/>
-      <c r="C2" s="132"/>
-      <c r="D2" s="132"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="127"/>
+      <c r="D2" s="127"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
-      <c r="I2" s="99"/>
+      <c r="I2" s="90"/>
       <c r="J2" s="6"/>
       <c r="K2" s="7"/>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="59" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="104" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="104"/>
       <c r="D3" s="105"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118"/>
-      <c r="J3" s="118"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
+      <c r="J3" s="133"/>
       <c r="K3" s="9"/>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" ht="13.2">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="133" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" s="134"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="118"/>
-      <c r="I4" s="118"/>
-      <c r="J4" s="118"/>
+      <c r="B4" s="134" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="135"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="133"/>
+      <c r="I4" s="133"/>
+      <c r="J4" s="133"/>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" s="77" customFormat="1" ht="26.4">
-      <c r="A5" s="68" t="s">
+    <row r="5" spans="1:11" s="71" customFormat="1" ht="26.4">
+      <c r="A5" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="136" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="139"/>
-      <c r="I5" s="139"/>
-      <c r="J5" s="139"/>
-      <c r="K5" s="76"/>
+      <c r="B5" s="129" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="130"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="132"/>
+      <c r="I5" s="132"/>
+      <c r="J5" s="132"/>
+      <c r="K5" s="70"/>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A6" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="88">
-        <f>COUNTIF(I12:I17,"Pass")</f>
-        <v>1</v>
+      <c r="B6" s="81">
+        <f>COUNTIF(I:I,"Pass")</f>
+        <v>2</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIF(I10:I736,"Pending")</f>
+        <f>COUNTIF(I:I,"Pending")</f>
         <v>0</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="118"/>
-      <c r="I6" s="118"/>
-      <c r="J6" s="118"/>
+      <c r="H6" s="133"/>
+      <c r="I6" s="133"/>
+      <c r="J6" s="133"/>
       <c r="K6" s="9"/>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1" thickBot="1">
       <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="89">
-        <f>COUNTIF(I12:I17,"Fail")</f>
+      <c r="B7" s="82">
+        <f>COUNTIF(I:I,"Fail")</f>
         <v>1</v>
       </c>
       <c r="C7" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="64">
-        <f>COUNTA(A12:A17) -15</f>
-        <v>-11</v>
-      </c>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="118"/>
-      <c r="I7" s="118"/>
-      <c r="J7" s="118"/>
+      <c r="D7" s="60">
+        <f>COUNTIF(A:A, "TC*")</f>
+        <v>3</v>
+      </c>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="133"/>
+      <c r="I7" s="133"/>
+      <c r="J7" s="133"/>
       <c r="K7" s="9"/>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="119"/>
-      <c r="B8" s="119"/>
-      <c r="C8" s="119"/>
-      <c r="D8" s="119"/>
+      <c r="A8" s="128"/>
+      <c r="B8" s="128"/>
+      <c r="C8" s="128"/>
+      <c r="D8" s="128"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
-      <c r="I8" s="100"/>
-      <c r="J8" s="100"/>
+      <c r="I8" s="91"/>
+      <c r="J8" s="91"/>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" s="79" customFormat="1" ht="12" customHeight="1">
-      <c r="A9" s="120" t="s">
+    <row r="9" spans="1:11" s="73" customFormat="1" ht="12" customHeight="1">
+      <c r="A9" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="122" t="s">
+      <c r="B9" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="120" t="s">
+      <c r="C9" s="114" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="124" t="s">
+      <c r="D9" s="115" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="126"/>
-      <c r="H9" s="130" t="s">
+      <c r="E9" s="116"/>
+      <c r="F9" s="116"/>
+      <c r="G9" s="117"/>
+      <c r="H9" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="121" t="s">
+      <c r="I9" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="121" t="s">
+      <c r="J9" s="106" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="78"/>
+      <c r="K9" s="72"/>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="121"/>
-      <c r="B10" s="123"/>
-      <c r="C10" s="121"/>
-      <c r="D10" s="127"/>
-      <c r="E10" s="128"/>
-      <c r="F10" s="128"/>
-      <c r="G10" s="129"/>
-      <c r="H10" s="127"/>
-      <c r="I10" s="121"/>
-      <c r="J10" s="121"/>
+      <c r="A10" s="106"/>
+      <c r="B10" s="125"/>
+      <c r="C10" s="106"/>
+      <c r="D10" s="118"/>
+      <c r="E10" s="119"/>
+      <c r="F10" s="119"/>
+      <c r="G10" s="120"/>
+      <c r="H10" s="118"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" s="80" customFormat="1" ht="15">
-      <c r="A11" s="108"/>
-      <c r="B11" s="108"/>
-      <c r="C11" s="108"/>
-      <c r="D11" s="108"/>
-      <c r="E11" s="108"/>
-      <c r="F11" s="108"/>
-      <c r="G11" s="108"/>
-      <c r="H11" s="108"/>
-      <c r="I11" s="108"/>
-      <c r="J11" s="109"/>
-    </row>
-    <row r="12" spans="1:11" s="4" customFormat="1" ht="13.2">
-      <c r="A12" s="110" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="111"/>
-      <c r="C12" s="111"/>
-      <c r="D12" s="111"/>
-      <c r="E12" s="111"/>
-      <c r="F12" s="111"/>
-      <c r="G12" s="111"/>
-      <c r="H12" s="111"/>
-      <c r="I12" s="111"/>
-      <c r="J12" s="112"/>
-    </row>
-    <row r="13" spans="1:11" s="4" customFormat="1" ht="83.4" customHeight="1" outlineLevel="1">
-      <c r="A13" s="84" t="s">
+    <row r="11" spans="1:11" s="74" customFormat="1" ht="15">
+      <c r="A11" s="122"/>
+      <c r="B11" s="122"/>
+      <c r="C11" s="122"/>
+      <c r="D11" s="122"/>
+      <c r="E11" s="122"/>
+      <c r="F11" s="122"/>
+      <c r="G11" s="122"/>
+      <c r="H11" s="122"/>
+      <c r="I11" s="122"/>
+      <c r="J11" s="123"/>
+    </row>
+    <row r="12" spans="1:11" s="4" customFormat="1" ht="13.2" customHeight="1">
+      <c r="A12" s="109" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="110"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="111"/>
+    </row>
+    <row r="13" spans="1:11" s="4" customFormat="1" ht="96" customHeight="1" outlineLevel="1">
+      <c r="A13" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="90" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="83" t="s">
-        <v>67</v>
+      <c r="B13" s="83" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="77" t="s">
+        <v>49</v>
       </c>
       <c r="D13" s="113" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" s="114"/>
-      <c r="F13" s="114"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="140" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="76"/>
+      <c r="H13" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="I13" s="83" t="s">
+      <c r="I13" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" s="75"/>
+    </row>
+    <row r="14" spans="1:11" s="4" customFormat="1" ht="94.8" customHeight="1" outlineLevel="1">
+      <c r="A14" s="78"/>
+      <c r="B14" s="83" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="77" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="113" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
+      <c r="G14" s="76"/>
+      <c r="H14" s="94" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="77" t="s">
+        <v>3</v>
+      </c>
+      <c r="J14" s="75"/>
+    </row>
+    <row r="15" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" outlineLevel="1">
+      <c r="A15" s="109" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="110"/>
+      <c r="C15" s="110"/>
+      <c r="D15" s="110"/>
+      <c r="E15" s="110"/>
+      <c r="F15" s="110"/>
+      <c r="G15" s="110"/>
+      <c r="H15" s="110"/>
+      <c r="I15" s="110"/>
+      <c r="J15" s="111"/>
+    </row>
+    <row r="16" spans="1:11" s="4" customFormat="1" ht="96.6" customHeight="1" outlineLevel="1">
+      <c r="A16" s="78" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="83" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="87" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="107" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="84" t="s">
+        <v>44</v>
+      </c>
+      <c r="I16" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="J16" s="75" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" s="4" customFormat="1" ht="108" customHeight="1" outlineLevel="1">
+      <c r="A17" s="78"/>
+      <c r="B17" s="83" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="87" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" s="107" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="84" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="81"/>
-    </row>
-    <row r="14" spans="1:11" s="4" customFormat="1" ht="13.2" outlineLevel="1">
-      <c r="A14" s="110" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="111"/>
-      <c r="C14" s="111"/>
-      <c r="D14" s="95"/>
-      <c r="E14" s="95"/>
-      <c r="F14" s="95"/>
-      <c r="G14" s="95"/>
-      <c r="H14" s="95"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="96"/>
-    </row>
-    <row r="15" spans="1:11" s="4" customFormat="1" ht="81.599999999999994" customHeight="1" outlineLevel="1">
-      <c r="A15" s="84" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="94" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="94" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="115" t="s">
-        <v>70</v>
-      </c>
-      <c r="E15" s="114"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="82"/>
-      <c r="H15" s="91" t="s">
+      <c r="J17" s="75" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="16.2" customHeight="1">
+      <c r="A18" s="109" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="110"/>
+      <c r="C18" s="110"/>
+      <c r="D18" s="110"/>
+      <c r="E18" s="110"/>
+      <c r="F18" s="110"/>
+      <c r="G18" s="110"/>
+      <c r="H18" s="110"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="111"/>
+    </row>
+    <row r="19" spans="1:10" ht="94.8" customHeight="1">
+      <c r="A19" s="78" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="77" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="107" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="108"/>
+      <c r="F19" s="108"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="84" t="s">
         <v>44</v>
       </c>
-      <c r="I15" s="83" t="s">
-        <v>3</v>
-      </c>
-      <c r="J15" s="81"/>
-    </row>
-    <row r="16" spans="1:11" s="4" customFormat="1" ht="13.2" outlineLevel="1">
-      <c r="A16" s="116"/>
-      <c r="B16" s="117"/>
-      <c r="C16" s="117"/>
-      <c r="D16" s="95"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="95"/>
-      <c r="G16" s="95"/>
-      <c r="H16" s="95"/>
-      <c r="I16" s="95"/>
-      <c r="J16" s="96"/>
-    </row>
-    <row r="17" spans="1:10" s="4" customFormat="1" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A17" s="84"/>
-      <c r="B17" s="101"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="106"/>
-      <c r="E17" s="107"/>
-      <c r="F17" s="107"/>
-      <c r="G17" s="82"/>
-      <c r="H17" s="91"/>
-      <c r="I17" s="83"/>
-      <c r="J17" s="81"/>
-    </row>
-    <row r="18" spans="1:10" ht="12" customHeight="1"/>
-    <row r="19" spans="1:10" ht="12" customHeight="1"/>
+      <c r="I19" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="J19" s="75" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+    </row>
     <row r="20" spans="1:10" ht="12" customHeight="1"/>
     <row r="21" spans="1:10" ht="12" customHeight="1"/>
     <row r="22" spans="1:10" ht="12" customHeight="1"/>
@@ -2538,32 +2893,35 @@
     <row r="54" ht="12" customHeight="1"/>
     <row r="55" ht="12" customHeight="1"/>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="26">
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H7:J7"/>
     <mergeCell ref="B3:D3"/>
+    <mergeCell ref="H4:J4"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:G10"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="A11:J11"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -2571,336 +2929,433 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F6884C4-AFEC-4BBC-9DC8-80B5528C1C8F}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.8" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="42.109375" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" customWidth="1"/>
-    <col min="7" max="7" width="18.44140625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="17.109375" customWidth="1"/>
-    <col min="9" max="9" width="9" style="93"/>
-    <col min="10" max="10" width="18" style="92" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.109375" style="1" customWidth="1"/>
+    <col min="4" max="5" width="8.77734375" style="1"/>
+    <col min="6" max="6" width="23.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" style="1" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" style="86"/>
+    <col min="10" max="10" width="18" style="103" customWidth="1"/>
+    <col min="11" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
-      <c r="I1" s="99"/>
+      <c r="I1" s="90"/>
       <c r="J1" s="6"/>
       <c r="K1" s="7"/>
     </row>
     <row r="2" spans="1:11" s="2" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
       <c r="A2" s="7"/>
-      <c r="B2" s="132"/>
-      <c r="C2" s="132"/>
-      <c r="D2" s="132"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="127"/>
+      <c r="D2" s="127"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
-      <c r="I2" s="99"/>
+      <c r="I2" s="90"/>
       <c r="J2" s="6"/>
       <c r="K2" s="7"/>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A3" s="63" t="s">
-        <v>36</v>
+      <c r="A3" s="59" t="s">
+        <v>93</v>
       </c>
       <c r="B3" s="104" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="104"/>
       <c r="D3" s="105"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118"/>
-      <c r="J3" s="118"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
+      <c r="J3" s="133"/>
       <c r="K3" s="9"/>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" ht="13.2">
-      <c r="A4" s="68" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="133" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="134"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="118"/>
-      <c r="I4" s="118"/>
-      <c r="J4" s="118"/>
+      <c r="A4" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="134" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="135"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="133"/>
+      <c r="I4" s="133"/>
+      <c r="J4" s="133"/>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" s="77" customFormat="1" ht="26.4">
-      <c r="A5" s="68" t="s">
+    <row r="5" spans="1:11" s="71" customFormat="1" ht="26.4">
+      <c r="A5" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="136" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="139"/>
-      <c r="I5" s="139"/>
-      <c r="J5" s="139"/>
-      <c r="K5" s="76"/>
+      <c r="B5" s="129" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="130"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="132"/>
+      <c r="I5" s="132"/>
+      <c r="J5" s="132"/>
+      <c r="K5" s="70"/>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A6" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="88">
-        <f>COUNTIF(I12:I17,"Pass")</f>
-        <v>1</v>
+      <c r="B6" s="81">
+        <f>COUNTIF(I:I,"Pass")</f>
+        <v>2</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIF(I10:I736,"Pending")</f>
+        <f>COUNTIF(I:I,"Pending")</f>
         <v>0</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="118"/>
-      <c r="I6" s="118"/>
-      <c r="J6" s="118"/>
+      <c r="H6" s="133"/>
+      <c r="I6" s="133"/>
+      <c r="J6" s="133"/>
       <c r="K6" s="9"/>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1" thickBot="1">
       <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="89">
-        <f>COUNTIF(I12:I17,"Fail")</f>
-        <v>2</v>
+      <c r="B7" s="82">
+        <f>COUNTIF(I:I,"Fail")</f>
+        <v>3</v>
       </c>
       <c r="C7" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="64">
-        <f>COUNTA(A12:A17) -15</f>
-        <v>-9</v>
-      </c>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="118"/>
-      <c r="I7" s="118"/>
-      <c r="J7" s="118"/>
+      <c r="D7" s="60">
+        <f>COUNTIF(A:A, "TC*")</f>
+        <v>5</v>
+      </c>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="133"/>
+      <c r="I7" s="133"/>
+      <c r="J7" s="133"/>
       <c r="K7" s="9"/>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="119"/>
-      <c r="B8" s="119"/>
-      <c r="C8" s="119"/>
-      <c r="D8" s="119"/>
+      <c r="A8" s="128"/>
+      <c r="B8" s="128"/>
+      <c r="C8" s="128"/>
+      <c r="D8" s="128"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
-      <c r="I8" s="100"/>
-      <c r="J8" s="100"/>
+      <c r="I8" s="91"/>
+      <c r="J8" s="91"/>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" s="79" customFormat="1" ht="12" customHeight="1">
-      <c r="A9" s="120" t="s">
+    <row r="9" spans="1:11" s="73" customFormat="1" ht="12" customHeight="1">
+      <c r="A9" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="122" t="s">
+      <c r="B9" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="120" t="s">
+      <c r="C9" s="114" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="124" t="s">
+      <c r="D9" s="115" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="126"/>
-      <c r="H9" s="130" t="s">
+      <c r="E9" s="116"/>
+      <c r="F9" s="116"/>
+      <c r="G9" s="117"/>
+      <c r="H9" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="121" t="s">
+      <c r="I9" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="121" t="s">
+      <c r="J9" s="106" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="78"/>
+      <c r="K9" s="72"/>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="121"/>
-      <c r="B10" s="123"/>
-      <c r="C10" s="121"/>
-      <c r="D10" s="127"/>
-      <c r="E10" s="128"/>
-      <c r="F10" s="128"/>
-      <c r="G10" s="129"/>
-      <c r="H10" s="127"/>
-      <c r="I10" s="121"/>
-      <c r="J10" s="121"/>
+      <c r="A10" s="106"/>
+      <c r="B10" s="125"/>
+      <c r="C10" s="106"/>
+      <c r="D10" s="118"/>
+      <c r="E10" s="119"/>
+      <c r="F10" s="119"/>
+      <c r="G10" s="120"/>
+      <c r="H10" s="118"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" s="80" customFormat="1" ht="15">
-      <c r="A11" s="108"/>
-      <c r="B11" s="108"/>
-      <c r="C11" s="108"/>
-      <c r="D11" s="108"/>
-      <c r="E11" s="108"/>
-      <c r="F11" s="108"/>
-      <c r="G11" s="108"/>
-      <c r="H11" s="108"/>
-      <c r="I11" s="108"/>
-      <c r="J11" s="109"/>
+    <row r="11" spans="1:11" s="102" customFormat="1" ht="15">
+      <c r="A11" s="122"/>
+      <c r="B11" s="122"/>
+      <c r="C11" s="122"/>
+      <c r="D11" s="122"/>
+      <c r="E11" s="122"/>
+      <c r="F11" s="122"/>
+      <c r="G11" s="122"/>
+      <c r="H11" s="122"/>
+      <c r="I11" s="122"/>
+      <c r="J11" s="123"/>
     </row>
     <row r="12" spans="1:11" s="4" customFormat="1" ht="13.2">
-      <c r="A12" s="110" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="111"/>
-      <c r="C12" s="111"/>
-      <c r="D12" s="111"/>
-      <c r="E12" s="111"/>
-      <c r="F12" s="111"/>
-      <c r="G12" s="111"/>
-      <c r="H12" s="111"/>
-      <c r="I12" s="111"/>
-      <c r="J12" s="112"/>
-    </row>
-    <row r="13" spans="1:11" s="4" customFormat="1" ht="92.4" outlineLevel="1">
-      <c r="A13" s="84" t="s">
+      <c r="A12" s="109" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="110"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="111"/>
+    </row>
+    <row r="13" spans="1:11" s="4" customFormat="1" ht="83.4" customHeight="1" outlineLevel="1">
+      <c r="A13" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="90" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="83" t="s">
-        <v>50</v>
+      <c r="B13" s="83" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="77" t="s">
+        <v>63</v>
       </c>
       <c r="D13" s="113" t="s">
-        <v>52</v>
-      </c>
-      <c r="E13" s="114"/>
-      <c r="F13" s="114"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="140" t="s">
+        <v>82</v>
+      </c>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="76"/>
+      <c r="H13" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="I13" s="83" t="s">
+      <c r="I13" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="J13" s="75"/>
+    </row>
+    <row r="14" spans="1:11" s="4" customFormat="1" ht="13.2" customHeight="1" outlineLevel="1">
+      <c r="A14" s="109" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="110"/>
+      <c r="C14" s="110"/>
+      <c r="D14" s="110"/>
+      <c r="E14" s="110"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="110"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="111"/>
+    </row>
+    <row r="15" spans="1:11" s="4" customFormat="1" ht="81.599999999999994" customHeight="1" outlineLevel="1">
+      <c r="A15" s="78" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="87" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="87" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="107" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="84" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="75"/>
+    </row>
+    <row r="16" spans="1:11" s="4" customFormat="1" ht="79.8" customHeight="1" outlineLevel="1">
+      <c r="A16" s="78"/>
+      <c r="B16" s="87" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="87" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="107" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="84" t="s">
+        <v>68</v>
+      </c>
+      <c r="I16" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="J13" s="81"/>
-    </row>
-    <row r="14" spans="1:11" s="4" customFormat="1" ht="13.2" customHeight="1" outlineLevel="1">
-      <c r="A14" s="110" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="111"/>
-      <c r="C14" s="111"/>
-      <c r="D14" s="111"/>
-      <c r="E14" s="111"/>
-      <c r="F14" s="111"/>
-      <c r="G14" s="111"/>
-      <c r="H14" s="111"/>
-      <c r="I14" s="111"/>
-      <c r="J14" s="112"/>
-    </row>
-    <row r="15" spans="1:11" s="4" customFormat="1" ht="94.8" customHeight="1" outlineLevel="1">
-      <c r="A15" s="84" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="90" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="94" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="115" t="s">
-        <v>53</v>
-      </c>
-      <c r="E15" s="114"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="82"/>
-      <c r="H15" s="91" t="s">
-        <v>44</v>
-      </c>
-      <c r="I15" s="83" t="s">
+      <c r="J16" s="75"/>
+    </row>
+    <row r="17" spans="1:10" ht="12" customHeight="1">
+      <c r="A17" s="109" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="110"/>
+      <c r="C17" s="110"/>
+      <c r="D17" s="110"/>
+      <c r="E17" s="110"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="110"/>
+      <c r="H17" s="110"/>
+      <c r="I17" s="110"/>
+      <c r="J17" s="111"/>
+    </row>
+    <row r="18" spans="1:10" ht="107.4" customHeight="1">
+      <c r="A18" s="78" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="99" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="107" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="108"/>
+      <c r="F18" s="108"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="84" t="s">
+        <v>68</v>
+      </c>
+      <c r="I18" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="J15" s="81" t="e" vm="1">
+      <c r="J18" s="75" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="4" customFormat="1" ht="13.2" customHeight="1" outlineLevel="1">
-      <c r="A16" s="110" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="111"/>
-      <c r="C16" s="111"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="111"/>
-      <c r="G16" s="111"/>
-      <c r="H16" s="111"/>
-      <c r="I16" s="111"/>
-      <c r="J16" s="112"/>
-    </row>
-    <row r="17" spans="1:10" s="4" customFormat="1" ht="97.2" customHeight="1" outlineLevel="1">
-      <c r="A17" s="84" t="s">
-        <v>2</v>
-      </c>
-      <c r="B17" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="83" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="115" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" s="107"/>
-      <c r="F17" s="107"/>
-      <c r="G17" s="82"/>
-      <c r="H17" s="91" t="s">
-        <v>44</v>
-      </c>
-      <c r="I17" s="83" t="s">
+    <row r="19" spans="1:10" ht="12" customHeight="1">
+      <c r="A19" s="109" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="110"/>
+      <c r="C19" s="110"/>
+      <c r="D19" s="110"/>
+      <c r="E19" s="110"/>
+      <c r="F19" s="110"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="111"/>
+    </row>
+    <row r="20" spans="1:10" ht="107.4" customHeight="1">
+      <c r="A20" s="78" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="77" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="99" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="107" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="108"/>
+      <c r="F20" s="108"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="84" t="s">
+        <v>68</v>
+      </c>
+      <c r="I20" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="J17" s="81" t="e" vm="2">
+      <c r="J20" s="75" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="12" customHeight="1"/>
-    <row r="19" spans="1:10" ht="12" customHeight="1"/>
-    <row r="20" spans="1:10" ht="12" customHeight="1"/>
-    <row r="21" spans="1:10" ht="12" customHeight="1"/>
-    <row r="22" spans="1:10" ht="12" customHeight="1"/>
+    <row r="21" spans="1:10" ht="12" customHeight="1">
+      <c r="A21" s="109" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="110"/>
+      <c r="C21" s="110"/>
+      <c r="D21" s="110"/>
+      <c r="E21" s="110"/>
+      <c r="F21" s="110"/>
+      <c r="G21" s="110"/>
+      <c r="H21" s="110"/>
+      <c r="I21" s="110"/>
+      <c r="J21" s="111"/>
+    </row>
+    <row r="22" spans="1:10" ht="107.4" customHeight="1">
+      <c r="A22" s="78" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="77" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="99" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="107" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="108"/>
+      <c r="F22" s="108"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="100">
+        <v>45661</v>
+      </c>
+      <c r="I22" s="77" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="75" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+    </row>
     <row r="23" spans="1:10" ht="12" customHeight="1"/>
     <row r="24" spans="1:10" ht="12" customHeight="1"/>
     <row r="25" spans="1:10" ht="12" customHeight="1"/>
@@ -2933,35 +3388,38 @@
     <row r="52" ht="12" customHeight="1"/>
     <row r="53" ht="12" customHeight="1"/>
     <row r="54" ht="12" customHeight="1"/>
-    <row r="55" ht="12" customHeight="1"/>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="A8:D8"/>
+  <mergeCells count="29">
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="D22:F22"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A12:J12"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="H6:J6"/>
     <mergeCell ref="H7:J7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="B1:D2"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="J9:J10"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="D18:F18"/>
     <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:G10"/>
   </mergeCells>
-  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -2971,10 +3429,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="3" max="3" width="22.77734375" customWidth="1"/>
-    <col min="7" max="7" width="18.77734375" customWidth="1"/>
+    <col min="1" max="2" width="8.77734375" style="1"/>
+    <col min="3" max="3" width="22.77734375" style="1" customWidth="1"/>
+    <col min="4" max="6" width="8.77734375" style="1"/>
+    <col min="7" max="7" width="18.77734375" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22.2">
@@ -2997,7 +3458,7 @@
       <c r="F2" s="17"/>
       <c r="G2" s="18"/>
     </row>
-    <row r="3" spans="1:7" ht="13.8">
+    <row r="3" spans="1:7">
       <c r="B3" s="19" t="s">
         <v>10</v>
       </c>
@@ -3007,17 +3468,17 @@
       <c r="F3" s="17"/>
       <c r="G3" s="18"/>
     </row>
-    <row r="4" spans="1:7" ht="13.8">
+    <row r="4" spans="1:7">
       <c r="B4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="98"/>
+      <c r="C4" s="89"/>
       <c r="D4" s="19"/>
       <c r="E4" s="19"/>
       <c r="F4" s="19"/>
       <c r="G4" s="19"/>
     </row>
-    <row r="5" spans="1:7" ht="13.8">
+    <row r="5" spans="1:7">
       <c r="A5" s="19"/>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3026,7 +3487,7 @@
       <c r="F5" s="19"/>
       <c r="G5" s="19"/>
     </row>
-    <row r="6" spans="1:7" ht="13.8">
+    <row r="6" spans="1:7">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
@@ -3037,84 +3498,101 @@
     </row>
     <row r="7" spans="1:7" ht="26.4">
       <c r="A7" s="19"/>
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="55" t="s">
+      <c r="D7" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="54" t="s">
+      <c r="F7" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="56" t="s">
+      <c r="G7" s="52" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="65" customFormat="1" ht="26.4">
-      <c r="A8" s="69"/>
-      <c r="B8" s="70">
+    <row r="8" spans="1:7" s="101" customFormat="1" ht="26.4">
+      <c r="A8" s="64"/>
+      <c r="B8" s="65">
         <v>1</v>
       </c>
-      <c r="C8" s="71" t="str">
+      <c r="C8" s="66" t="str">
         <f>'Module Register'!B4</f>
         <v>REG100 - User Registration</v>
       </c>
-      <c r="D8" s="72">
+      <c r="D8" s="67">
         <f>'Module Register'!B6</f>
+        <v>2</v>
+      </c>
+      <c r="E8" s="66">
+        <f>'Module Register'!B7</f>
         <v>1</v>
       </c>
-      <c r="E8" s="71">
-        <f>'Module Register'!B7</f>
-        <v>2</v>
-      </c>
-      <c r="F8" s="71">
+      <c r="F8" s="66">
         <f>'Module Register'!D6</f>
         <v>0</v>
       </c>
-      <c r="G8" s="72">
+      <c r="G8" s="67">
         <f>'Module Register'!D7</f>
-        <v>-9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="13.8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="22.2" customHeight="1">
       <c r="A9" s="19"/>
-      <c r="B9" s="32"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="33"/>
-    </row>
-    <row r="10" spans="1:7" ht="13.8">
+      <c r="B9" s="96">
+        <v>2</v>
+      </c>
+      <c r="C9" s="37" t="str">
+        <f>'Module Login'!B4</f>
+        <v>AUTH - User Login</v>
+      </c>
+      <c r="D9" s="97">
+        <f>'Module Login'!B6</f>
+        <v>2</v>
+      </c>
+      <c r="E9" s="97">
+        <f>'Module Login'!B7</f>
+        <v>3</v>
+      </c>
+      <c r="F9" s="97">
+        <f>'Module Login'!D6</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="98">
+        <f>'Module Login'!D7</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="19"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="58" t="s">
+      <c r="B10" s="53"/>
+      <c r="C10" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="59">
+      <c r="D10" s="55">
         <f>SUM(D6:D9)</f>
-        <v>1</v>
-      </c>
-      <c r="E10" s="59">
+        <v>4</v>
+      </c>
+      <c r="E10" s="55">
         <f>SUM(E6:E9)</f>
-        <v>2</v>
-      </c>
-      <c r="F10" s="59">
+        <v>4</v>
+      </c>
+      <c r="F10" s="55">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="60">
+      <c r="G10" s="56">
         <f>SUM(G6:G9)</f>
-        <v>-9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="13.8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="19"/>
       <c r="B11" s="20"/>
       <c r="C11" s="19"/>
@@ -3123,7 +3601,7 @@
       <c r="F11" s="22"/>
       <c r="G11" s="22"/>
     </row>
-    <row r="12" spans="1:7" ht="13.8">
+    <row r="12" spans="1:7">
       <c r="A12" s="19"/>
       <c r="B12" s="19"/>
       <c r="C12" s="19" t="s">
@@ -3132,14 +3610,14 @@
       <c r="D12" s="19"/>
       <c r="E12" s="23">
         <f>(D10+E10)*100/G10</f>
-        <v>-33.333333333333336</v>
+        <v>100</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="24"/>
     </row>
-    <row r="13" spans="1:7" ht="13.8">
+    <row r="13" spans="1:7">
       <c r="A13" s="19"/>
       <c r="B13" s="19"/>
       <c r="C13" s="19" t="s">
@@ -3148,7 +3626,7 @@
       <c r="D13" s="19"/>
       <c r="E13" s="23">
         <f>D10*100/G10</f>
-        <v>-11.111111111111111</v>
+        <v>50</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>22</v>

</xml_diff>